<commit_message>
style: Use darker gray for disabled cells in Excel opinion sheet
</commit_message>
<xml_diff>
--- a/Excels/PresetLayerOpinionSheet.xlsx
+++ b/Excels/PresetLayerOpinionSheet.xlsx
@@ -66,11 +66,11 @@
     <font>
       <name val="Meiryo"/>
       <i val="1"/>
-      <color rgb="009CA3AF"/>
+      <color rgb="004B5563"/>
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -117,6 +117,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFFF"/>
         <bgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D1D5DB"/>
+        <bgColor rgb="00D1D5DB"/>
       </patternFill>
     </fill>
   </fills>
@@ -172,7 +178,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>

</xml_diff>